<commit_message>
Still doing simulation base
</commit_message>
<xml_diff>
--- a/Simulation_Bases/I_2.xlsx
+++ b/Simulation_Bases/I_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://insalyonfrance-my.sharepoint.com/personal/sserranose_insa-lyon_fr/Documents/Bureau/Code/Panda_pipes/Simulation_Bases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{E77B25B0-7A6E-4DE9-85DC-B34A0D4FB441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D039E07-E9E3-4AF0-A54D-79703EAA2C95}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="8_{E77B25B0-7A6E-4DE9-85DC-B34A0D4FB441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32BDB49A-74F1-4B1C-92A2-86913948CAFC}"/>
   <bookViews>
-    <workbookView xWindow="-24045" yWindow="1200" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{DE24DEA2-80CA-4F40-BB26-7FB15C90EEDE}"/>
+    <workbookView xWindow="-28920" yWindow="-1470" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{DE24DEA2-80CA-4F40-BB26-7FB15C90EEDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet_1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Sheet_3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet_4" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet_5" sheetId="7" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="8" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="9" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
   <si>
     <t>N1</t>
   </si>
@@ -105,16 +108,64 @@
     <t>k_mm</t>
   </si>
   <si>
-    <t>p_flow_bar</t>
-  </si>
-  <si>
-    <t>plift_bar</t>
-  </si>
-  <si>
     <t>t_flow_k</t>
   </si>
   <si>
     <t>Consumer</t>
+  </si>
+  <si>
+    <t>Vtot</t>
+  </si>
+  <si>
+    <t>T_hot_init</t>
+  </si>
+  <si>
+    <t>T_cold_init</t>
+  </si>
+  <si>
+    <t>v_hot_fraction</t>
+  </si>
+  <si>
+    <t>UA_loss</t>
+  </si>
+  <si>
+    <t>UA_interface</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refrigerant </t>
+  </si>
+  <si>
+    <t>R134a</t>
+  </si>
+  <si>
+    <t>dT_water</t>
+  </si>
+  <si>
+    <t>eta_s</t>
+  </si>
+  <si>
+    <t>Fuel_type</t>
+  </si>
+  <si>
+    <t>Nominal_efficiency</t>
+  </si>
+  <si>
+    <t>Emission_factor</t>
+  </si>
+  <si>
+    <t>cost_constant</t>
+  </si>
+  <si>
+    <t>P_out_design</t>
+  </si>
+  <si>
+    <t>P_lift_design</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>T_return</t>
   </si>
 </sst>
 </file>
@@ -677,7 +728,7 @@
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -803,6 +854,200 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D144322-F7F2-4697-908B-50708F72AA90}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFE886A9-53DB-4678-9CB5-0CCEEDB8F47A}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6286BB6-2EBB-4C5D-91DF-6BB4D064C440}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <v>0.95</v>
+      </c>
+      <c r="C4">
+        <v>0.95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C132E5D2-F4BE-4B9C-A1CE-6EFDC3AAB10A}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -810,38 +1055,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFE886A9-53DB-4678-9CB5-0CCEEDB8F47A}">
-  <dimension ref="A1:B4"/>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA2311F4-3FFB-497E-8886-C1ED7F7302D8}">
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>